<commit_message>
add dosen & mhs  by excel
</commit_message>
<xml_diff>
--- a/public/templates/template_import_mahasiswa.xlsx
+++ b/public/templates/template_import_mahasiswa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\download\lms\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\lms\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AEC44F4-E0C1-4440-868F-6CFF23DD07B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F69B06-1A6C-4C3B-9187-80BDA5299C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,16 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>john@example.com</t>
+  </si>
+  <si>
+    <t>john</t>
+  </si>
+  <si>
+    <t>nim</t>
+  </si>
   <si>
     <t>nama</t>
   </si>
@@ -28,25 +37,19 @@
     <t>email</t>
   </si>
   <si>
+    <t>program studi</t>
+  </si>
+  <si>
     <t>semester</t>
   </si>
   <si>
-    <t>john@example.com</t>
-  </si>
-  <si>
-    <t>nim</t>
-  </si>
-  <si>
-    <t>program studi</t>
-  </si>
-  <si>
-    <t>john</t>
+    <t>angkatan</t>
   </si>
   <si>
     <t>phone</t>
   </si>
   <si>
-    <t>teknik somputer</t>
+    <t>teknik komputer</t>
   </si>
 </sst>
 </file>
@@ -100,8 +103,12 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -405,64 +412,68 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="4" max="4" width="17.140625" customWidth="1"/>
-    <col min="5" max="5" width="20.42578125" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" customWidth="1"/>
+    <col min="2" max="2" width="18.26953125" customWidth="1"/>
+    <col min="3" max="3" width="17.7265625" customWidth="1"/>
+    <col min="4" max="4" width="17.1796875" customWidth="1"/>
+    <col min="5" max="5" width="20.453125" customWidth="1"/>
+    <col min="6" max="6" width="18.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="E1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>7</v>
       </c>
+      <c r="G1" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>22231231</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="2">
         <v>2</v>
       </c>
       <c r="F2">
+        <v>2026</v>
+      </c>
+      <c r="G2">
         <v>92233</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B3" s="1"/>
-      <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B4" s="1"/>
-      <c r="E4" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
memperbaiki semua fitur, termasuk tugas quizz, nilai dan chat
</commit_message>
<xml_diff>
--- a/public/templates/template_import_mahasiswa.xlsx
+++ b/public/templates/template_import_mahasiswa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\download\lms\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\lms\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AEC44F4-E0C1-4440-868F-6CFF23DD07B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F69B06-1A6C-4C3B-9187-80BDA5299C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,16 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>john@example.com</t>
+  </si>
+  <si>
+    <t>john</t>
+  </si>
+  <si>
+    <t>nim</t>
+  </si>
   <si>
     <t>nama</t>
   </si>
@@ -28,25 +37,19 @@
     <t>email</t>
   </si>
   <si>
+    <t>program studi</t>
+  </si>
+  <si>
     <t>semester</t>
   </si>
   <si>
-    <t>john@example.com</t>
-  </si>
-  <si>
-    <t>nim</t>
-  </si>
-  <si>
-    <t>program studi</t>
-  </si>
-  <si>
-    <t>john</t>
+    <t>angkatan</t>
   </si>
   <si>
     <t>phone</t>
   </si>
   <si>
-    <t>teknik somputer</t>
+    <t>teknik komputer</t>
   </si>
 </sst>
 </file>
@@ -100,8 +103,12 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -405,64 +412,68 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="4" max="4" width="17.140625" customWidth="1"/>
-    <col min="5" max="5" width="20.42578125" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" customWidth="1"/>
+    <col min="2" max="2" width="18.26953125" customWidth="1"/>
+    <col min="3" max="3" width="17.7265625" customWidth="1"/>
+    <col min="4" max="4" width="17.1796875" customWidth="1"/>
+    <col min="5" max="5" width="20.453125" customWidth="1"/>
+    <col min="6" max="6" width="18.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="E1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>7</v>
       </c>
+      <c r="G1" s="3" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>22231231</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" s="2">
         <v>2</v>
       </c>
       <c r="F2">
+        <v>2026</v>
+      </c>
+      <c r="G2">
         <v>92233</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B3" s="1"/>
-      <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B4" s="1"/>
-      <c r="E4" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>